<commit_message>
Release v2.0 - SmartStudentManager
Version 2.0 of SmartStudent Manager.

This update introduces a dashboard to provide a clear overview of student fee status, including total students, paid, and unpaid counts.

The notification system has been improved for better handling of SMS alerts.

Enhancements:
- Dashboard with fee status summary
- Improved notification workflow
- Better user interface and feedback messages

This version builds on the Excel-based system and focuses on improving usability for front-office staff.
</commit_message>
<xml_diff>
--- a/studentdata.xlsx
+++ b/studentdata.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,12 +496,12 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Sem 5 Fee</t>
+          <t>Sem 1 Fee</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Sem 5 Result</t>
+          <t>Sem 1 Result</t>
         </is>
       </c>
     </row>
@@ -689,16 +689,8 @@
           <t>2025-05-02</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>32323</t>
-        </is>
-      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -960,6 +952,152 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>162</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1623</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ezra</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ganapathi</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>roja</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>hjjdjdjdjjdjdjdjdjdjdjjdjd</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>polavarapuezra22@gmail.com</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>7675009869</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>12365478789</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2000-03-09</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>mca</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2022-08-12</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>25000</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>162</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1623</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ezra</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ganapathi</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>roja</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>hjjdjdjdjjdjdjdjdjdjdjjdjd</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>polavarapuezra22@gmail.com</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>7675009869</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>12365478789</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2000-03-09</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>mca</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2022-08-12</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>25000</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>